<commit_message>
split rule status into success/issue reported/skipped/execution error + uniform excel styling
</commit_message>
<xml_diff>
--- a/resources/templates/report-template.xlsx
+++ b/resources/templates/report-template.xlsx
@@ -88,7 +88,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -115,11 +115,44 @@
         <color rgb="002E5F55"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -154,6 +187,7 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -677,7 +711,7 @@
           <t>Conformance Details</t>
         </is>
       </c>
-      <c r="B1" s="12" t="n"/>
+      <c r="B1" s="18" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="13" t="inlineStr">
@@ -703,14 +737,13 @@
       </c>
       <c r="B4" s="14" t="n"/>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
           <t>Standards Details</t>
         </is>
       </c>
-      <c r="B6" s="12" t="n"/>
+      <c r="B6" s="18" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="13" t="inlineStr">
@@ -2252,7 +2285,7 @@
       </c>
       <c r="G1" s="17" t="inlineStr">
         <is>
-          <t>Reason for Skip</t>
+          <t>Reason</t>
         </is>
       </c>
     </row>

</xml_diff>